<commit_message>
📊 Actualizar LIDERES_ACTIVOS.xlsx — 08-04-2026, 12:08:16 p. m.
</commit_message>
<xml_diff>
--- a/datos/LIDERES_ACTIVOS.xlsx
+++ b/datos/LIDERES_ACTIVOS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos de Mes/ABRIL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D82D248F-0C7E-43E6-A584-32824881D94A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{D0049C2E-1A73-460B-8324-CB8B99BDBA5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0F9AA18-015D-49B2-9C8E-02D8FF1AFC0F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{218CA180-2924-470B-AC01-76D4BF6A104A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="16">
   <si>
     <t>Lider</t>
   </si>
@@ -78,9 +78,6 @@
   </si>
   <si>
     <t>Raúl Alejandro Bustos Aguilera</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paula García Steembecker </t>
   </si>
   <si>
     <t xml:space="preserve">Glenda Patricia Martínez Ortiz </t>
@@ -493,7 +490,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0282BA47-F3BB-4FCA-AF70-814913F551CE}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.6640625" bestFit="1" customWidth="1"/>
@@ -611,17 +608,6 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>